<commit_message>
Completed Step 2: Verified sorting, pull-to-refresh, random country navigation, and updated test spreadsheet
</commit_message>
<xml_diff>
--- a/CountryExplorer/docs/CountryExplorer_Test_Plan_and_Results.xlsx
+++ b/CountryExplorer/docs/CountryExplorer_Test_Plan_and_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\CountryExplorer\CountryExplorer\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7A9AAE4-F61F-4246-B597-CEBE71AC7F24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C768E7B-91BE-44C3-822F-3E2385496E4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8232" yWindow="372" windowWidth="14892" windowHeight="11592" xr2:uid="{EEEDD6F8-1991-4E89-8E54-7088AD5D3B07}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="69">
   <si>
     <t>Test Case ID:</t>
   </si>
@@ -189,6 +189,63 @@
   </si>
   <si>
     <t>Test Plan &amp; Results Table</t>
+  </si>
+  <si>
+    <t>Extension</t>
+  </si>
+  <si>
+    <t>TC-12</t>
+  </si>
+  <si>
+    <t>TC-13</t>
+  </si>
+  <si>
+    <t>TC-14</t>
+  </si>
+  <si>
+    <t>TC-15</t>
+  </si>
+  <si>
+    <t>TC-16</t>
+  </si>
+  <si>
+    <t>TC-17</t>
+  </si>
+  <si>
+    <t>Multi-Criteria Sorting</t>
+  </si>
+  <si>
+    <t>Pull-to-Refresh</t>
+  </si>
+  <si>
+    <t>Random Selection</t>
+  </si>
+  <si>
+    <t>Dataset Coverage</t>
+  </si>
+  <si>
+    <t>Change Sort By picker between Name (A-Z/Z-A) and Population (High-Low/Low-High).</t>
+  </si>
+  <si>
+    <t>Swipe/drag down on the main CollectionView.</t>
+  </si>
+  <si>
+    <t>Click the toolbar 🎲 Random button.</t>
+  </si>
+  <si>
+    <t>Filter through all regions (Africa, Americas, Asia, Europe, Oceania).</t>
+  </si>
+  <si>
+    <t>List reorders immediately according to selected property and direction.</t>
+  </si>
+  <si>
+    <t>RefreshView triggers, invokes LoadCountryDataAsync(), and updates the UI.</t>
+  </si>
+  <si>
+    <t>Picks a country at random and navigates directly to CountryDetailsPage.</t>
+  </si>
+  <si>
+    <t>Every region displays flag cards with population and capital details.</t>
   </si>
 </sst>
 </file>
@@ -650,7 +707,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1975C7E-753C-4B91-BFE2-B2D2AF63B542}">
-  <dimension ref="B3:G17"/>
+  <dimension ref="B3:G23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
@@ -852,19 +909,109 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="C15" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="C16" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
         <v>16</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B18" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B19" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B20" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B21" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B22" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B23" s="1" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>